<commit_message>
Added a locally hosted website for the visualization of the order informations
</commit_message>
<xml_diff>
--- a/FAT_INSTALL Plan Worksheet.xlsx
+++ b/FAT_INSTALL Plan Worksheet.xlsx
@@ -1440,7 +1440,11 @@
         </is>
       </c>
       <c r="B24" s="45" t="n"/>
-      <c r="C24" s="45" t="n"/>
+      <c r="C24" s="45" t="inlineStr">
+        <is>
+          <t>12/01/2021</t>
+        </is>
+      </c>
       <c r="D24" s="29" t="inlineStr">
         <is>
           <t>Confirm order from ZRU to ZNRA: Get confirming order to XXX with FAT &amp; delivery expectations</t>
@@ -1453,7 +1457,7 @@
       </c>
       <c r="F24" s="28" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G24" s="28" t="inlineStr">
@@ -1461,7 +1465,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H24" s="29" t="n"/>
+      <c r="H24" s="29" t="inlineStr">
+        <is>
+          <t>OC received from ZRX 12/01/2021</t>
+        </is>
+      </c>
       <c r="I24" s="30" t="inlineStr">
         <is>
           <t>Purchase Order</t>
@@ -1709,7 +1717,11 @@
         </is>
       </c>
       <c r="B31" s="49" t="n"/>
-      <c r="C31" s="49" t="n"/>
+      <c r="C31" s="49" t="inlineStr">
+        <is>
+          <t>12/6/2021</t>
+        </is>
+      </c>
       <c r="D31" s="24" t="inlineStr">
         <is>
           <t>Shipment of system</t>
@@ -1722,7 +1734,7 @@
       </c>
       <c r="F31" s="40" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G31" s="40" t="inlineStr">
@@ -1730,7 +1742,11 @@
           <t>Task 7</t>
         </is>
       </c>
-      <c r="H31" s="24" t="n"/>
+      <c r="H31" s="24" t="inlineStr">
+        <is>
+          <t>Shipped (tracking 1ZV357A50442428615)</t>
+        </is>
+      </c>
       <c r="I31" s="41" t="inlineStr">
         <is>
           <t>Shipping Documents</t>

</xml_diff>